<commit_message>
Added some python files and little updates.
</commit_message>
<xml_diff>
--- a/Codes/Scripts/Test/test.xlsx
+++ b/Codes/Scripts/Test/test.xlsx
@@ -602,40 +602,40 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="B2" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="C2" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.675</v>
+        <v>0.54</v>
       </c>
       <c r="E2" t="n">
         <v>125</v>
       </c>
       <c r="F2" t="n">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="G2" t="n">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="L2" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -644,13 +644,13 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P2" t="n">
-        <v>8.342207999999999</v>
+        <v>8.350272</v>
       </c>
       <c r="Q2" t="n">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="R2" t="n">
         <v>10</v>
@@ -659,16 +659,16 @@
         <v>8</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0234991774648</v>
+        <v>0.0233901176471</v>
       </c>
       <c r="U2" t="n">
         <v>244</v>
       </c>
       <c r="V2" t="n">
-        <v>83.9295774648</v>
+        <v>83.99719887960001</v>
       </c>
       <c r="W2" t="n">
-        <v>1.88169014085</v>
+        <v>1.87675070028</v>
       </c>
       <c r="X2" t="n">
         <v>1</v>
@@ -683,13 +683,13 @@
         <v>1</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.0721722247475</v>
+        <v>0.051390781407</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.0759707628921</v>
+        <v>0.05710086823</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -704,7 +704,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>saed05rvt_base_ss0p675v125c</t>
+          <t>saed05rvt_base_ss0p540v125c</t>
         </is>
       </c>
     </row>

</xml_diff>